<commit_message>
Popravek - Ibrahim Čaušević
</commit_message>
<xml_diff>
--- a/CausevicIbrahim/projektnaNaloga/CausevicIbrahim.xlsx
+++ b/CausevicIbrahim/projektnaNaloga/CausevicIbrahim.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Domaca naloga 7\projekt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\CausevicIbrahim\alma2026racunalnistvoOblak\CausevicIbrahim\projektnaNaloga\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{447F21D1-9AFF-4CD7-A02C-38DA3C8BFC0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97C7C379-DB51-4909-ACD4-A03035AE6BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -424,7 +424,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -449,14 +449,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="14">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -645,11 +639,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -659,16 +673,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -678,34 +683,67 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1481,99 +1519,99 @@
   <sheetData>
     <row r="1" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="B2" s="12">
+      <c r="B2" s="15">
         <v>1</v>
       </c>
-      <c r="C2" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="5" t="s">
+      <c r="C2" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="14" t="s">
         <v>53</v>
       </c>
       <c r="O2" s="9"/>
     </row>
     <row r="3" spans="2:16" ht="225" x14ac:dyDescent="0.25">
-      <c r="B3" s="14"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="5" t="s">
+      <c r="B3" s="17"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="L3" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="N3" s="14" t="s">
         <v>55</v>
       </c>
       <c r="O3" s="9"/>
-      <c r="P3" s="9" t="s">
+      <c r="P3" s="6" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="4" spans="2:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="B4" s="16">
+      <c r="B4" s="11">
         <v>1</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="14" t="s">
         <v>47</v>
       </c>
       <c r="F4" s="4"/>
@@ -1586,115 +1624,115 @@
       <c r="M4" s="4"/>
       <c r="N4" s="4"/>
       <c r="O4" s="9"/>
-      <c r="P4" s="10" t="s">
+      <c r="P4" s="7" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B5" s="16">
+      <c r="B5" s="26">
         <v>2</v>
       </c>
-      <c r="C5" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="D5" s="5" t="s">
+      <c r="C5" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="D5" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="19" t="s">
         <v>18</v>
       </c>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
-      <c r="N5" s="7"/>
+      <c r="N5" s="5"/>
       <c r="O5" s="9"/>
-      <c r="P5" s="11" t="s">
+      <c r="P5" s="8" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="6" spans="2:16" ht="180" x14ac:dyDescent="0.25">
-      <c r="B6" s="16"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="5" t="s">
+      <c r="B6" s="26"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4" t="s">
+      <c r="E6" s="19"/>
+      <c r="F6" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" s="19" t="s">
         <v>62</v>
       </c>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
       <c r="M6" s="4"/>
-      <c r="N6" s="7"/>
+      <c r="N6" s="5"/>
       <c r="O6" s="9"/>
     </row>
     <row r="7" spans="2:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="B7" s="16">
+      <c r="B7" s="11">
         <v>2</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="H7" s="4"/>
+      <c r="H7" s="14"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
       <c r="M7" s="4"/>
-      <c r="N7" s="7"/>
+      <c r="N7" s="5"/>
       <c r="O7" s="9"/>
     </row>
     <row r="8" spans="2:16" ht="285" x14ac:dyDescent="0.25">
-      <c r="B8" s="16"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="6" t="s">
+      <c r="B8" s="11"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4" t="s">
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14" t="s">
         <v>68</v>
       </c>
       <c r="I8" s="4"/>
@@ -1702,80 +1740,80 @@
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
       <c r="M8" s="4"/>
-      <c r="N8" s="7"/>
+      <c r="N8" s="5"/>
       <c r="O8" s="9"/>
     </row>
     <row r="9" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B9" s="16">
+      <c r="B9" s="26">
         <v>3</v>
       </c>
-      <c r="C9" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="D9" s="6" t="s">
+      <c r="C9" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="D9" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="19" t="s">
         <v>26</v>
       </c>
       <c r="J9" s="4"/>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
-      <c r="N9" s="7"/>
+      <c r="N9" s="5"/>
       <c r="O9" s="9"/>
     </row>
     <row r="10" spans="2:16" ht="120" x14ac:dyDescent="0.25">
-      <c r="B10" s="16"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="6" t="s">
+      <c r="B10" s="26"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="19" t="s">
         <v>75</v>
       </c>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
-      <c r="N10" s="7"/>
+      <c r="N10" s="5"/>
       <c r="O10" s="9"/>
     </row>
     <row r="11" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B11" s="16">
+      <c r="B11" s="11">
         <v>4</v>
       </c>
-      <c r="C11" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="D11" s="6" t="s">
+      <c r="C11" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="14" t="s">
         <v>28</v>
       </c>
       <c r="F11" s="4"/>
@@ -1786,16 +1824,16 @@
       <c r="K11" s="4"/>
       <c r="L11" s="4"/>
       <c r="M11" s="4"/>
-      <c r="N11" s="7"/>
+      <c r="N11" s="5"/>
       <c r="O11" s="9"/>
     </row>
     <row r="12" spans="2:16" ht="195" x14ac:dyDescent="0.25">
-      <c r="B12" s="16"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="6" t="s">
+      <c r="B12" s="11"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="14" t="s">
         <v>77</v>
       </c>
       <c r="F12" s="4"/>
@@ -1806,26 +1844,26 @@
       <c r="K12" s="4"/>
       <c r="L12" s="4"/>
       <c r="M12" s="4"/>
-      <c r="N12" s="7"/>
+      <c r="N12" s="5"/>
       <c r="O12" s="9"/>
     </row>
     <row r="13" spans="2:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="B13" s="16">
+      <c r="B13" s="11">
         <v>4</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="14" t="s">
         <v>30</v>
       </c>
       <c r="H13" s="4"/>
@@ -1834,18 +1872,18 @@
       <c r="K13" s="4"/>
       <c r="L13" s="4"/>
       <c r="M13" s="4"/>
-      <c r="N13" s="7"/>
+      <c r="N13" s="5"/>
       <c r="O13" s="9"/>
     </row>
     <row r="14" spans="2:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="B14" s="16"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="6" t="s">
+      <c r="B14" s="11"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4" t="s">
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14" t="s">
         <v>79</v>
       </c>
       <c r="H14" s="4"/>
@@ -1854,26 +1892,26 @@
       <c r="K14" s="4"/>
       <c r="L14" s="4"/>
       <c r="M14" s="4"/>
-      <c r="N14" s="7"/>
+      <c r="N14" s="5"/>
       <c r="O14" s="9"/>
     </row>
     <row r="15" spans="2:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="B15" s="16">
+      <c r="B15" s="11">
         <v>5</v>
       </c>
-      <c r="C15" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="D15" s="6" t="s">
+      <c r="C15" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="D15" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="F15" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="14" t="s">
         <v>32</v>
       </c>
       <c r="H15" s="4"/>
@@ -1882,22 +1920,22 @@
       <c r="K15" s="4"/>
       <c r="L15" s="4"/>
       <c r="M15" s="4"/>
-      <c r="N15" s="7"/>
+      <c r="N15" s="5"/>
       <c r="O15" s="9"/>
     </row>
     <row r="16" spans="2:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="B16" s="16"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="6" t="s">
+      <c r="B16" s="11"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="14" t="s">
         <v>84</v>
       </c>
       <c r="H16" s="4"/>
@@ -1906,20 +1944,20 @@
       <c r="K16" s="4"/>
       <c r="L16" s="4"/>
       <c r="M16" s="4"/>
-      <c r="N16" s="7"/>
+      <c r="N16" s="5"/>
       <c r="O16" s="9"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="16">
+      <c r="B17" s="11">
         <v>5</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="C17" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="14" t="s">
         <v>78</v>
       </c>
       <c r="F17" s="4"/>
@@ -1930,14 +1968,14 @@
       <c r="K17" s="4"/>
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
-      <c r="N17" s="7"/>
+      <c r="N17" s="5"/>
       <c r="O17" s="9"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B18" s="16"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="4"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="14"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1946,29 +1984,29 @@
       <c r="K18" s="4"/>
       <c r="L18" s="4"/>
       <c r="M18" s="4"/>
-      <c r="N18" s="7"/>
+      <c r="N18" s="5"/>
       <c r="O18" s="9"/>
     </row>
     <row r="19" spans="2:15" ht="45" x14ac:dyDescent="0.25">
-      <c r="B19" s="16">
+      <c r="B19" s="11">
         <v>6</v>
       </c>
-      <c r="C19" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="D19" s="6" t="s">
+      <c r="C19" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="D19" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="H19" s="14" t="s">
         <v>93</v>
       </c>
       <c r="I19" s="4"/>
@@ -1976,42 +2014,42 @@
       <c r="K19" s="4"/>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
-      <c r="N19" s="7"/>
+      <c r="N19" s="5"/>
       <c r="O19" s="9"/>
     </row>
     <row r="20" spans="2:15" ht="120" x14ac:dyDescent="0.25">
-      <c r="B20" s="16"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="6" t="s">
+      <c r="B20" s="11"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
-      <c r="N20" s="7"/>
+      <c r="N20" s="5"/>
       <c r="O20" s="9"/>
     </row>
     <row r="21" spans="2:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="B21" s="16">
+      <c r="B21" s="11">
         <v>7</v>
       </c>
-      <c r="C21" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="D21" s="6" t="s">
+      <c r="C21" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="D21" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="14" t="s">
         <v>95</v>
       </c>
       <c r="F21" s="4"/>
@@ -2022,16 +2060,16 @@
       <c r="K21" s="4"/>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
-      <c r="N21" s="7"/>
+      <c r="N21" s="5"/>
       <c r="O21" s="9"/>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B22" s="16"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="6" t="s">
+      <c r="B22" s="11"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="E22" s="4"/>
+      <c r="E22" s="14"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -2040,29 +2078,29 @@
       <c r="K22" s="4"/>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
-      <c r="N22" s="7"/>
+      <c r="N22" s="5"/>
       <c r="O22" s="9"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B23" s="16">
+      <c r="B23" s="11">
         <v>7</v>
       </c>
-      <c r="C23" s="17" t="s">
+      <c r="C23" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="G23" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="H23" s="4" t="s">
+      <c r="H23" s="14" t="s">
         <v>96</v>
       </c>
       <c r="I23" s="4"/>
@@ -2070,17 +2108,17 @@
       <c r="K23" s="4"/>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
-      <c r="N23" s="7"/>
+      <c r="N23" s="5"/>
       <c r="O23" s="9"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B24" s="16">
+      <c r="B24" s="11">
         <v>8</v>
       </c>
-      <c r="C24" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="D24" s="6" t="s">
+      <c r="C24" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="D24" s="20" t="s">
         <v>40</v>
       </c>
       <c r="E24" s="4"/>
@@ -2092,17 +2130,17 @@
       <c r="K24" s="4"/>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
-      <c r="N24" s="7"/>
+      <c r="N24" s="5"/>
       <c r="O24" s="9"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B25" s="18">
+      <c r="B25" s="21">
         <v>8</v>
       </c>
-      <c r="C25" s="19" t="s">
+      <c r="C25" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="20" t="s">
         <v>40</v>
       </c>
       <c r="E25" s="4"/>
@@ -2114,17 +2152,17 @@
       <c r="K25" s="4"/>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
-      <c r="N25" s="7"/>
-      <c r="O25" s="9"/>
+      <c r="N25" s="5"/>
+      <c r="O25" s="10"/>
     </row>
     <row r="26" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="20">
+      <c r="B26" s="23">
         <v>9</v>
       </c>
-      <c r="C26" s="21" t="s">
-        <v>0</v>
-      </c>
-      <c r="D26" s="8" t="s">
+      <c r="C26" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="D26" s="25" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>